<commit_message>
initial provider suite, payer suite that simulates a client
</commit_message>
<xml_diff>
--- a/lib/davinci_dtr_test_kit/requirements/hl7.fhir.us.davinci-dtr_2.2.0_requirements.xlsx
+++ b/lib/davinci_dtr_test_kit/requirements/hl7.fhir.us.davinci-dtr_2.2.0_requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-dtr-test-kit/lib/davinci_dtr_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A095CAB-3DAA-FD41-945E-8DA720F4CF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5844B4E5-697F-8A43-B73C-CEA81DB8CF3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1960" windowWidth="34560" windowHeight="20380" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -3156,9 +3156,6 @@
     <t>https://hl7.org/fhir/us/davinci-dtr/2.2.0/en/specification.html#ci-c-spec-121</t>
   </si>
   <si>
-    <t>If the launch context did not include Coverages, a QuestionnaireResponse or a Request or Encounter, the DTR app‚ÄØ**SHALL** either‚ÄØgenerate an error or‚ÄØallow the user to search to find one to use as context for the DTR session.</t>
-  </si>
-  <si>
     <t>spec-122</t>
   </si>
   <si>
@@ -3586,6 +3583,9 @@
   </si>
   <si>
     <t>If dependencies are such that a steady state cannot be reached (e.g., an item that is enabled causes a value to be set which causes a different item to be enabled, that then disables the first item...), then the Questionnaire SHALL be treated as erroneous and attempts at automatic population SHALL end, with the user being informed of that.</t>
+  </si>
+  <si>
+    <t>If the launch context did not include Coverages, a QuestionnaireResponse or a Request or Encounter, the DTR app **SHALL** either generate an error or allow the user to search to find one to use as context for the DTR session.</t>
   </si>
 </sst>
 </file>
@@ -4468,6 +4468,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W216"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4589,7 +4590,7 @@
         <v>ci-c-conf-1</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="85" x14ac:dyDescent="0.2">
@@ -4620,7 +4621,7 @@
         <v>ci-c-conf-2</v>
       </c>
       <c r="P3" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="51" x14ac:dyDescent="0.2">
@@ -4651,10 +4652,10 @@
         <v>ci-c-conf-3</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="119" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>92</v>
       </c>
@@ -4682,14 +4683,14 @@
         <v>ci-c-conf-4</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="7" t="s">
         <v>96</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -4713,7 +4714,7 @@
         <v>ci-c-conf-5</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="85" x14ac:dyDescent="0.2">
@@ -4744,10 +4745,10 @@
         <v>ci-c-conf-6</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="34" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>101</v>
       </c>
@@ -4775,10 +4776,10 @@
         <v>ci-c-conf-7</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" ht="102" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>104</v>
       </c>
@@ -4806,10 +4807,10 @@
         <v>ci-c-conf-8</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>108</v>
       </c>
@@ -4837,10 +4838,10 @@
         <v>ci-c-conf-9</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" ht="170" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" ht="170" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>111</v>
       </c>
@@ -4868,10 +4869,10 @@
         <v>ci-c-conf-10</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>115</v>
       </c>
@@ -4899,7 +4900,7 @@
         <v>ci-c-conf-11</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="153" x14ac:dyDescent="0.2">
@@ -4930,7 +4931,7 @@
         <v>ci-c-conf-12</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="102" x14ac:dyDescent="0.2">
@@ -4961,7 +4962,7 @@
         <v>ci-c-conf-13</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="136" x14ac:dyDescent="0.2">
@@ -4992,7 +4993,7 @@
         <v>ci-c-conf-14</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="16" spans="1:23" ht="51" x14ac:dyDescent="0.2">
@@ -5023,10 +5024,10 @@
         <v>ci-c-conf-15</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>131</v>
       </c>
@@ -5054,10 +5055,10 @@
         <v>ci-c-opcn-1</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>134</v>
       </c>
@@ -5085,7 +5086,7 @@
         <v>ci-c-opcn-2</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -5116,7 +5117,7 @@
         <v>ci-c-oper-1</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="136" x14ac:dyDescent="0.2">
@@ -5147,10 +5148,10 @@
         <v>ci-c-oper-2</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>144</v>
       </c>
@@ -5178,7 +5179,7 @@
         <v>ci-c-oper-3</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -5209,10 +5210,10 @@
         <v>ci-c-oper-4</v>
       </c>
       <c r="P22" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>150</v>
       </c>
@@ -5240,7 +5241,7 @@
         <v>ci-c-oper-5</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -5271,14 +5272,14 @@
         <v>ci-c-oper-6</v>
       </c>
       <c r="P24" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="11" t="s">
         <v>157</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -5302,10 +5303,10 @@
         <v>ci-c-oper-7</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>159</v>
       </c>
@@ -5333,10 +5334,10 @@
         <v>ci-c-oper-8</v>
       </c>
       <c r="P26" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>162</v>
       </c>
@@ -5364,10 +5365,10 @@
         <v>ci-c-oper-9</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>165</v>
       </c>
@@ -5395,10 +5396,10 @@
         <v>ci-c-oper-10</v>
       </c>
       <c r="P28" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>168</v>
       </c>
@@ -5426,10 +5427,10 @@
         <v>ci-c-oper-11</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>171</v>
       </c>
@@ -5457,10 +5458,10 @@
         <v>ci-c-oper-12</v>
       </c>
       <c r="P30" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>174</v>
       </c>
@@ -5488,10 +5489,10 @@
         <v>ci-c-oper-13</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>177</v>
       </c>
@@ -5519,10 +5520,10 @@
         <v>ci-c-oper-14</v>
       </c>
       <c r="P32" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>180</v>
       </c>
@@ -5550,10 +5551,10 @@
         <v>ci-c-oper-15</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
         <v>183</v>
       </c>
@@ -5581,10 +5582,10 @@
         <v>ci-c-oper-16</v>
       </c>
       <c r="P34" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
         <v>186</v>
       </c>
@@ -5612,10 +5613,10 @@
         <v>ci-c-oper-17</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>189</v>
       </c>
@@ -5643,10 +5644,10 @@
         <v>ci-c-oper-18</v>
       </c>
       <c r="P36" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>192</v>
       </c>
@@ -5674,7 +5675,7 @@
         <v>ci-c-oper-19</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="136" x14ac:dyDescent="0.2">
@@ -5705,10 +5706,10 @@
         <v>ci-c-oper-20</v>
       </c>
       <c r="P38" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
         <v>198</v>
       </c>
@@ -5736,14 +5737,14 @@
         <v>ci-c-prof-1</v>
       </c>
       <c r="P39" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="85" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="7" t="s">
         <v>202</v>
       </c>
       <c r="C40" s="8" t="s">
@@ -5767,7 +5768,7 @@
         <v>ci-c-prof-2</v>
       </c>
       <c r="P40" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -5798,10 +5799,10 @@
         <v>ci-c-sec-1</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
         <v>207</v>
       </c>
@@ -5829,10 +5830,10 @@
         <v>ci-c-sec-2</v>
       </c>
       <c r="P42" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
         <v>210</v>
       </c>
@@ -5860,10 +5861,10 @@
         <v>ci-c-sec-3</v>
       </c>
       <c r="P43" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
         <v>213</v>
       </c>
@@ -5891,7 +5892,7 @@
         <v>ci-c-sec-4</v>
       </c>
       <c r="P44" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -5922,10 +5923,10 @@
         <v>ci-c-sec-5</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
         <v>218</v>
       </c>
@@ -5953,10 +5954,10 @@
         <v>ci-c-sec-6</v>
       </c>
       <c r="P46" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
         <v>220</v>
       </c>
@@ -5984,7 +5985,7 @@
         <v>ci-c-sec-7</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="48" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -6015,10 +6016,10 @@
         <v>ci-c-sec-8</v>
       </c>
       <c r="P48" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>225</v>
       </c>
@@ -6046,10 +6047,10 @@
         <v>ci-c-sec-9</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>228</v>
       </c>
@@ -6077,10 +6078,10 @@
         <v>ci-c-sec-10</v>
       </c>
       <c r="P50" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>231</v>
       </c>
@@ -6108,10 +6109,10 @@
         <v>ci-c-spec-1</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>234</v>
       </c>
@@ -6139,10 +6140,10 @@
         <v>ci-c-spec-2</v>
       </c>
       <c r="P52" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>237</v>
       </c>
@@ -6170,7 +6171,7 @@
         <v>ci-c-spec-3</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -6201,10 +6202,10 @@
         <v>ci-c-spec-4</v>
       </c>
       <c r="P54" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="55" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>243</v>
       </c>
@@ -6232,10 +6233,10 @@
         <v>ci-c-spec-5</v>
       </c>
       <c r="P55" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>246</v>
       </c>
@@ -6263,7 +6264,7 @@
         <v>ci-c-spec-6</v>
       </c>
       <c r="P56" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="57" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -6294,10 +6295,10 @@
         <v>ci-c-spec-7</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
         <v>252</v>
       </c>
@@ -6325,10 +6326,10 @@
         <v>ci-c-spec-8</v>
       </c>
       <c r="P58" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
         <v>255</v>
       </c>
@@ -6356,10 +6357,10 @@
         <v>ci-c-spec-9</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
         <v>259</v>
       </c>
@@ -6387,7 +6388,7 @@
         <v>ci-c-spec-10</v>
       </c>
       <c r="P60" s="10" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="61" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -6418,10 +6419,10 @@
         <v>ci-c-spec-11</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
         <v>265</v>
       </c>
@@ -6449,10 +6450,10 @@
         <v>ci-c-spec-12</v>
       </c>
       <c r="P62" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>269</v>
       </c>
@@ -6480,14 +6481,14 @@
         <v>ci-c-spec-13</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="64" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="B64" s="11" t="s">
+      <c r="B64" s="7" t="s">
         <v>273</v>
       </c>
       <c r="C64" s="8" t="s">
@@ -6511,10 +6512,10 @@
         <v>ci-c-spec-14</v>
       </c>
       <c r="P64" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
         <v>275</v>
       </c>
@@ -6542,7 +6543,7 @@
         <v>ci-c-spec-15</v>
       </c>
       <c r="P65" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="66" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -6573,10 +6574,10 @@
         <v>ci-c-spec-16</v>
       </c>
       <c r="P66" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="67" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>281</v>
       </c>
@@ -6604,10 +6605,10 @@
         <v>ci-c-spec-17</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
         <v>284</v>
       </c>
@@ -6635,7 +6636,7 @@
         <v>ci-c-spec-18</v>
       </c>
       <c r="P68" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="69" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -6666,7 +6667,7 @@
         <v>ci-c-spec-19</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="70" spans="1:16" ht="119" x14ac:dyDescent="0.2">
@@ -6697,10 +6698,10 @@
         <v>ci-c-spec-20</v>
       </c>
       <c r="P70" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
         <v>293</v>
       </c>
@@ -6728,10 +6729,10 @@
         <v>ci-c-spec-21</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
         <v>296</v>
       </c>
@@ -6759,10 +6760,10 @@
         <v>ci-c-spec-22</v>
       </c>
       <c r="P72" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="73" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
         <v>299</v>
       </c>
@@ -6790,10 +6791,10 @@
         <v>ci-c-spec-23</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="74" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
         <v>302</v>
       </c>
@@ -6821,14 +6822,14 @@
         <v>ci-c-spec-24</v>
       </c>
       <c r="P74" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="75" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="B75" s="7" t="s">
+      <c r="B75" s="11" t="s">
         <v>306</v>
       </c>
       <c r="C75" s="8" t="s">
@@ -6852,10 +6853,10 @@
         <v>ci-c-spec-25</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="76" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
         <v>308</v>
       </c>
@@ -6883,10 +6884,10 @@
         <v>ci-c-spec-26</v>
       </c>
       <c r="P76" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="77" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
         <v>311</v>
       </c>
@@ -6914,10 +6915,10 @@
         <v>ci-c-spec-27</v>
       </c>
       <c r="P77" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="78" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>314</v>
       </c>
@@ -6945,10 +6946,10 @@
         <v>ci-c-spec-28</v>
       </c>
       <c r="P78" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="79" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>317</v>
       </c>
@@ -6976,10 +6977,10 @@
         <v>ci-c-spec-29</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="80" spans="1:16" ht="187" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" ht="187" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
         <v>320</v>
       </c>
@@ -7007,10 +7008,10 @@
         <v>ci-c-spec-30</v>
       </c>
       <c r="P80" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>323</v>
       </c>
@@ -7038,10 +7039,10 @@
         <v>ci-c-spec-31</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="82" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>326</v>
       </c>
@@ -7069,10 +7070,10 @@
         <v>ci-c-spec-32</v>
       </c>
       <c r="P82" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="83" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
         <v>329</v>
       </c>
@@ -7100,10 +7101,10 @@
         <v>ci-c-spec-33</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="84" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
         <v>332</v>
       </c>
@@ -7131,7 +7132,7 @@
         <v>ci-c-spec-34</v>
       </c>
       <c r="P84" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="85" spans="1:16" ht="119" x14ac:dyDescent="0.2">
@@ -7162,10 +7163,10 @@
         <v>ci-c-spec-35</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
         <v>338</v>
       </c>
@@ -7193,10 +7194,10 @@
         <v>ci-c-spec-36</v>
       </c>
       <c r="P86" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="87" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
         <v>341</v>
       </c>
@@ -7224,10 +7225,10 @@
         <v>ci-c-spec-37</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="88" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
         <v>344</v>
       </c>
@@ -7255,10 +7256,10 @@
         <v>ci-c-spec-38</v>
       </c>
       <c r="P88" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="89" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
         <v>347</v>
       </c>
@@ -7286,10 +7287,10 @@
         <v>ci-c-spec-39</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="90" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
         <v>350</v>
       </c>
@@ -7317,10 +7318,10 @@
         <v>ci-c-spec-40</v>
       </c>
       <c r="P90" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="91" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
         <v>353</v>
       </c>
@@ -7348,10 +7349,10 @@
         <v>ci-c-spec-41</v>
       </c>
       <c r="P91" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="92" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
         <v>356</v>
       </c>
@@ -7379,10 +7380,10 @@
         <v>ci-c-spec-42</v>
       </c>
       <c r="P92" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="93" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
         <v>359</v>
       </c>
@@ -7410,7 +7411,7 @@
         <v>ci-c-spec-43</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="94" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -7441,10 +7442,10 @@
         <v>ci-c-spec-44</v>
       </c>
       <c r="P94" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="95" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="7" t="s">
         <v>365</v>
       </c>
@@ -7472,7 +7473,7 @@
         <v>ci-c-spec-45</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="96" spans="1:16" ht="119" x14ac:dyDescent="0.2">
@@ -7503,7 +7504,7 @@
         <v>ci-c-spec-46</v>
       </c>
       <c r="P96" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="97" spans="1:16" ht="153" x14ac:dyDescent="0.2">
@@ -7534,10 +7535,10 @@
         <v>ci-c-spec-47</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="98" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="7" t="s">
         <v>373</v>
       </c>
@@ -7565,7 +7566,7 @@
         <v>ci-c-spec-48</v>
       </c>
       <c r="P98" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="99" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -7596,10 +7597,10 @@
         <v>ci-c-spec-49</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="100" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" s="7" t="s">
         <v>379</v>
       </c>
@@ -7627,10 +7628,10 @@
         <v>ci-c-spec-50</v>
       </c>
       <c r="P100" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="101" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" s="7" t="s">
         <v>382</v>
       </c>
@@ -7658,10 +7659,10 @@
         <v>ci-c-spec-51</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="102" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" s="7" t="s">
         <v>384</v>
       </c>
@@ -7689,10 +7690,10 @@
         <v>ci-c-spec-52</v>
       </c>
       <c r="P102" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="103" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="7" t="s">
         <v>387</v>
       </c>
@@ -7720,10 +7721,10 @@
         <v>ci-c-spec-53</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="104" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="7" t="s">
         <v>390</v>
       </c>
@@ -7751,10 +7752,10 @@
         <v>ci-c-spec-54</v>
       </c>
       <c r="P104" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="105" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" s="7" t="s">
         <v>392</v>
       </c>
@@ -7782,10 +7783,10 @@
         <v>ci-c-spec-55</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="106" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" s="7" t="s">
         <v>395</v>
       </c>
@@ -7813,10 +7814,10 @@
         <v>ci-c-spec-56</v>
       </c>
       <c r="P106" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="107" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" s="7" t="s">
         <v>397</v>
       </c>
@@ -7844,10 +7845,10 @@
         <v>ci-c-spec-57</v>
       </c>
       <c r="P107" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="108" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="108" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
         <v>400</v>
       </c>
@@ -7875,7 +7876,7 @@
         <v>ci-c-spec-58</v>
       </c>
       <c r="P108" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="109" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -7906,7 +7907,7 @@
         <v>ci-c-spec-59</v>
       </c>
       <c r="P109" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="110" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -7937,10 +7938,10 @@
         <v>ci-c-spec-60</v>
       </c>
       <c r="P110" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="111" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="111" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="7" t="s">
         <v>409</v>
       </c>
@@ -7968,7 +7969,7 @@
         <v>ci-c-spec-61</v>
       </c>
       <c r="P111" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="112" spans="1:16" ht="238" x14ac:dyDescent="0.2">
@@ -7999,10 +8000,10 @@
         <v>ci-c-spec-62</v>
       </c>
       <c r="P112" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="113" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" s="7" t="s">
         <v>415</v>
       </c>
@@ -8030,7 +8031,7 @@
         <v>ci-c-spec-63</v>
       </c>
       <c r="P113" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="114" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -8061,7 +8062,7 @@
         <v>ci-c-spec-64</v>
       </c>
       <c r="P114" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="115" spans="1:16" ht="136" x14ac:dyDescent="0.2">
@@ -8092,7 +8093,7 @@
         <v>ci-c-spec-65</v>
       </c>
       <c r="P115" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="116" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -8123,7 +8124,7 @@
         <v>ci-c-spec-66</v>
       </c>
       <c r="P116" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="117" spans="1:16" ht="119" x14ac:dyDescent="0.2">
@@ -8134,7 +8135,7 @@
         <v>428</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D117" s="7" t="s">
         <v>26</v>
@@ -8154,7 +8155,7 @@
         <v>ci-c-spec-67</v>
       </c>
       <c r="P117" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="118" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -8185,10 +8186,10 @@
         <v>ci-c-spec-68</v>
       </c>
       <c r="P118" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="119" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="7" t="s">
         <v>432</v>
       </c>
@@ -8216,7 +8217,7 @@
         <v>ci-c-spec-69</v>
       </c>
       <c r="P119" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="120" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -8247,10 +8248,10 @@
         <v>ci-c-spec-70</v>
       </c>
       <c r="P120" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="121" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="7" t="s">
         <v>438</v>
       </c>
@@ -8278,7 +8279,7 @@
         <v>ci-c-spec-71</v>
       </c>
       <c r="P121" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="122" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -8309,7 +8310,7 @@
         <v>ci-c-spec-72</v>
       </c>
       <c r="P122" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="123" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -8340,7 +8341,7 @@
         <v>ci-c-spec-73</v>
       </c>
       <c r="P123" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="124" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -8371,10 +8372,10 @@
         <v>ci-c-spec-74</v>
       </c>
       <c r="P124" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="125" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="125" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="7" t="s">
         <v>450</v>
       </c>
@@ -8402,7 +8403,7 @@
         <v>ci-c-spec-75</v>
       </c>
       <c r="P125" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="126" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -8433,10 +8434,10 @@
         <v>ci-c-spec-76</v>
       </c>
       <c r="P126" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="127" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="7" t="s">
         <v>456</v>
       </c>
@@ -8464,7 +8465,7 @@
         <v>ci-c-spec-77</v>
       </c>
       <c r="P127" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="128" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -8495,7 +8496,7 @@
         <v>ci-c-spec-78</v>
       </c>
       <c r="P128" s="10" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="129" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -8526,10 +8527,10 @@
         <v>ci-c-spec-79</v>
       </c>
       <c r="P129" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="130" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="7" t="s">
         <v>465</v>
       </c>
@@ -8557,7 +8558,7 @@
         <v>ci-c-spec-80</v>
       </c>
       <c r="P130" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="131" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -8588,7 +8589,7 @@
         <v>ci-c-spec-81</v>
       </c>
       <c r="P131" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="132" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -8619,10 +8620,10 @@
         <v>ci-c-spec-82</v>
       </c>
       <c r="P132" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="133" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="7" t="s">
         <v>474</v>
       </c>
@@ -8650,10 +8651,10 @@
         <v>ci-c-spec-83</v>
       </c>
       <c r="P133" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="134" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="7" t="s">
         <v>477</v>
       </c>
@@ -8681,10 +8682,10 @@
         <v>ci-c-spec-84</v>
       </c>
       <c r="P134" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="135" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="7" t="s">
         <v>480</v>
       </c>
@@ -8712,10 +8713,10 @@
         <v>ci-c-spec-85</v>
       </c>
       <c r="P135" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="136" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="136" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" s="7" t="s">
         <v>483</v>
       </c>
@@ -8743,10 +8744,10 @@
         <v>ci-c-spec-86</v>
       </c>
       <c r="P136" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="137" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="137" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="7" t="s">
         <v>486</v>
       </c>
@@ -8774,10 +8775,10 @@
         <v>ci-c-spec-87</v>
       </c>
       <c r="P137" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="138" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="138" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" s="7" t="s">
         <v>489</v>
       </c>
@@ -8805,10 +8806,10 @@
         <v>ci-c-spec-88</v>
       </c>
       <c r="P138" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="139" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="139" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" s="7" t="s">
         <v>492</v>
       </c>
@@ -8836,10 +8837,10 @@
         <v>ci-c-spec-89</v>
       </c>
       <c r="P139" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="140" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="140" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="7" t="s">
         <v>495</v>
       </c>
@@ -8867,10 +8868,10 @@
         <v>ci-c-spec-90</v>
       </c>
       <c r="P140" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="141" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="141" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" s="7" t="s">
         <v>498</v>
       </c>
@@ -8898,10 +8899,10 @@
         <v>ci-c-spec-91</v>
       </c>
       <c r="P141" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="142" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="142" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="7" t="s">
         <v>501</v>
       </c>
@@ -8929,10 +8930,10 @@
         <v>ci-c-spec-92</v>
       </c>
       <c r="P142" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="143" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="143" spans="1:16" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="7" t="s">
         <v>504</v>
       </c>
@@ -8960,10 +8961,10 @@
         <v>ci-c-spec-93</v>
       </c>
       <c r="P143" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="144" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="144" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" s="7" t="s">
         <v>507</v>
       </c>
@@ -8991,10 +8992,10 @@
         <v>ci-c-spec-94</v>
       </c>
       <c r="P144" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="145" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="7" t="s">
         <v>510</v>
       </c>
@@ -9022,10 +9023,10 @@
         <v>ci-c-spec-95</v>
       </c>
       <c r="P145" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="146" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" s="7" t="s">
         <v>513</v>
       </c>
@@ -9053,10 +9054,10 @@
         <v>ci-c-spec-96</v>
       </c>
       <c r="P146" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="147" spans="1:16" ht="170" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="147" spans="1:16" ht="170" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" s="7" t="s">
         <v>516</v>
       </c>
@@ -9084,10 +9085,10 @@
         <v>ci-c-spec-97</v>
       </c>
       <c r="P147" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="148" spans="1:16" ht="119" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="148" spans="1:16" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="7" t="s">
         <v>519</v>
       </c>
@@ -9115,10 +9116,10 @@
         <v>ci-c-spec-98</v>
       </c>
       <c r="P148" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="149" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="149" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A149" s="7" t="s">
         <v>522</v>
       </c>
@@ -9146,10 +9147,10 @@
         <v>ci-c-spec-99</v>
       </c>
       <c r="P149" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="150" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="150" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" s="7" t="s">
         <v>525</v>
       </c>
@@ -9177,7 +9178,7 @@
         <v>ci-c-spec-100</v>
       </c>
       <c r="P150" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="151" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -9208,7 +9209,7 @@
         <v>ci-c-spec-101</v>
       </c>
       <c r="P151" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="152" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -9239,7 +9240,7 @@
         <v>ci-c-spec-102</v>
       </c>
       <c r="P152" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="153" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -9270,7 +9271,7 @@
         <v>ci-c-spec-103</v>
       </c>
       <c r="P153" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="154" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -9301,7 +9302,7 @@
         <v>ci-c-spec-104</v>
       </c>
       <c r="P154" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="155" spans="1:16" ht="119" x14ac:dyDescent="0.2">
@@ -9332,7 +9333,7 @@
         <v>ci-c-spec-105</v>
       </c>
       <c r="P155" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="156" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -9363,7 +9364,7 @@
         <v>ci-c-spec-106</v>
       </c>
       <c r="P156" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="157" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -9394,10 +9395,10 @@
         <v>ci-c-spec-107</v>
       </c>
       <c r="P157" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="158" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="158" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A158" s="7" t="s">
         <v>548</v>
       </c>
@@ -9425,7 +9426,7 @@
         <v>ci-c-spec-108</v>
       </c>
       <c r="P158" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="159" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -9456,10 +9457,10 @@
         <v>ci-c-spec-109</v>
       </c>
       <c r="P159" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="160" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="160" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" s="7" t="s">
         <v>554</v>
       </c>
@@ -9487,7 +9488,7 @@
         <v>ci-c-spec-110</v>
       </c>
       <c r="P160" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="161" spans="1:16" ht="136" x14ac:dyDescent="0.2">
@@ -9518,7 +9519,7 @@
         <v>ci-c-spec-111</v>
       </c>
       <c r="P161" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="162" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -9549,10 +9550,10 @@
         <v>ci-c-spec-112</v>
       </c>
       <c r="P162" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="163" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="163" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" s="7" t="s">
         <v>563</v>
       </c>
@@ -9580,10 +9581,10 @@
         <v>ci-c-spec-113</v>
       </c>
       <c r="P163" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="164" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="164" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" s="7" t="s">
         <v>566</v>
       </c>
@@ -9611,10 +9612,10 @@
         <v>ci-c-spec-114</v>
       </c>
       <c r="P164" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="165" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="165" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" s="7" t="s">
         <v>569</v>
       </c>
@@ -9642,7 +9643,7 @@
         <v>ci-c-spec-115</v>
       </c>
       <c r="P165" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="166" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -9673,7 +9674,7 @@
         <v>ci-c-spec-116</v>
       </c>
       <c r="P166" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="167" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -9704,10 +9705,10 @@
         <v>ci-c-spec-117</v>
       </c>
       <c r="P167" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="168" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="168" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" s="7" t="s">
         <v>578</v>
       </c>
@@ -9735,7 +9736,7 @@
         <v>ci-c-spec-118</v>
       </c>
       <c r="P168" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="169" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -9766,10 +9767,10 @@
         <v>ci-c-spec-119</v>
       </c>
       <c r="P169" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="170" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="170" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" s="7" t="s">
         <v>583</v>
       </c>
@@ -9797,7 +9798,7 @@
         <v>ci-c-spec-120</v>
       </c>
       <c r="P170" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="171" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -9808,7 +9809,7 @@
         <v>587</v>
       </c>
       <c r="C171" s="8" t="s">
-        <v>588</v>
+        <v>731</v>
       </c>
       <c r="D171" s="7" t="s">
         <v>26</v>
@@ -9828,18 +9829,18 @@
         <v>ci-c-spec-121</v>
       </c>
       <c r="P171" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="172" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="172" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="B172" s="7" t="s">
         <v>589</v>
       </c>
-      <c r="B172" s="7" t="s">
+      <c r="C172" s="8" t="s">
         <v>590</v>
-      </c>
-      <c r="C172" s="8" t="s">
-        <v>591</v>
       </c>
       <c r="D172" s="7" t="s">
         <v>26</v>
@@ -9859,18 +9860,18 @@
         <v>ci-c-spec-122</v>
       </c>
       <c r="P172" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="173" spans="1:16" ht="119" x14ac:dyDescent="0.2">
       <c r="A173" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="B173" s="7" t="s">
         <v>592</v>
       </c>
-      <c r="B173" s="7" t="s">
+      <c r="C173" s="8" t="s">
         <v>593</v>
-      </c>
-      <c r="C173" s="8" t="s">
-        <v>594</v>
       </c>
       <c r="D173" s="7" t="s">
         <v>26</v>
@@ -9890,18 +9891,18 @@
         <v>ci-c-spec-123</v>
       </c>
       <c r="P173" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="174" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="174" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A174" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="B174" s="7" t="s">
         <v>595</v>
       </c>
-      <c r="B174" s="7" t="s">
+      <c r="C174" s="8" t="s">
         <v>596</v>
-      </c>
-      <c r="C174" s="8" t="s">
-        <v>597</v>
       </c>
       <c r="D174" s="7" t="s">
         <v>29</v>
@@ -9921,18 +9922,18 @@
         <v>ci-c-spec-124</v>
       </c>
       <c r="P174" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="175" spans="1:16" ht="68" x14ac:dyDescent="0.2">
       <c r="A175" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="B175" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="B175" s="7" t="s">
+      <c r="C175" s="8" t="s">
         <v>599</v>
-      </c>
-      <c r="C175" s="8" t="s">
-        <v>600</v>
       </c>
       <c r="D175" s="7" t="s">
         <v>31</v>
@@ -9952,18 +9953,18 @@
         <v>ci-c-spec-125</v>
       </c>
       <c r="P175" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="176" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A176" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="B176" s="7" t="s">
         <v>601</v>
       </c>
-      <c r="B176" s="7" t="s">
+      <c r="C176" s="8" t="s">
         <v>602</v>
-      </c>
-      <c r="C176" s="8" t="s">
-        <v>603</v>
       </c>
       <c r="D176" s="7" t="s">
         <v>26</v>
@@ -9983,18 +9984,18 @@
         <v>ci-c-spec-126</v>
       </c>
       <c r="P176" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="177" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="177" spans="1:16" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="B177" s="7" t="s">
         <v>604</v>
       </c>
-      <c r="B177" s="7" t="s">
+      <c r="C177" s="8" t="s">
         <v>605</v>
-      </c>
-      <c r="C177" s="8" t="s">
-        <v>606</v>
       </c>
       <c r="D177" s="7" t="s">
         <v>30</v>
@@ -10014,18 +10015,18 @@
         <v>ci-c-spec-127</v>
       </c>
       <c r="P177" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="178" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="178" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="B178" s="7" t="s">
         <v>607</v>
       </c>
-      <c r="B178" s="7" t="s">
+      <c r="C178" s="8" t="s">
         <v>608</v>
-      </c>
-      <c r="C178" s="8" t="s">
-        <v>609</v>
       </c>
       <c r="D178" s="7" t="s">
         <v>26</v>
@@ -10045,18 +10046,18 @@
         <v>ci-c-spec-128</v>
       </c>
       <c r="P178" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="179" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="179" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="B179" s="7" t="s">
         <v>610</v>
       </c>
-      <c r="B179" s="7" t="s">
+      <c r="C179" s="8" t="s">
         <v>611</v>
-      </c>
-      <c r="C179" s="8" t="s">
-        <v>612</v>
       </c>
       <c r="D179" s="7" t="s">
         <v>30</v>
@@ -10076,18 +10077,18 @@
         <v>ci-c-spec-129</v>
       </c>
       <c r="P179" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="180" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="180" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="B180" s="7" t="s">
         <v>613</v>
       </c>
-      <c r="B180" s="7" t="s">
+      <c r="C180" s="8" t="s">
         <v>614</v>
-      </c>
-      <c r="C180" s="8" t="s">
-        <v>615</v>
       </c>
       <c r="D180" s="7" t="s">
         <v>26</v>
@@ -10107,18 +10108,18 @@
         <v>ci-c-spec-130</v>
       </c>
       <c r="P180" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="181" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="181" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A181" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="B181" s="7" t="s">
         <v>616</v>
       </c>
-      <c r="B181" s="7" t="s">
+      <c r="C181" s="8" t="s">
         <v>617</v>
-      </c>
-      <c r="C181" s="8" t="s">
-        <v>618</v>
       </c>
       <c r="D181" s="7" t="s">
         <v>30</v>
@@ -10138,18 +10139,18 @@
         <v>ci-c-spec-131</v>
       </c>
       <c r="P181" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="182" spans="1:16" ht="85" x14ac:dyDescent="0.2">
       <c r="A182" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="B182" s="7" t="s">
         <v>619</v>
       </c>
-      <c r="B182" s="7" t="s">
+      <c r="C182" s="8" t="s">
         <v>620</v>
-      </c>
-      <c r="C182" s="8" t="s">
-        <v>621</v>
       </c>
       <c r="D182" s="7" t="s">
         <v>26</v>
@@ -10169,18 +10170,18 @@
         <v>ci-c-spec-132</v>
       </c>
       <c r="P182" s="10" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="183" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="183" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" s="7" t="s">
+        <v>621</v>
+      </c>
+      <c r="B183" s="7" t="s">
         <v>622</v>
       </c>
-      <c r="B183" s="7" t="s">
+      <c r="C183" s="8" t="s">
         <v>623</v>
-      </c>
-      <c r="C183" s="8" t="s">
-        <v>624</v>
       </c>
       <c r="D183" s="7" t="s">
         <v>29</v>
@@ -10200,18 +10201,18 @@
         <v>ci-c-spec-133</v>
       </c>
       <c r="P183" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="184" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="184" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="B184" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="B184" s="7" t="s">
+      <c r="C184" s="8" t="s">
         <v>626</v>
-      </c>
-      <c r="C184" s="8" t="s">
-        <v>627</v>
       </c>
       <c r="D184" s="7" t="s">
         <v>29</v>
@@ -10231,18 +10232,18 @@
         <v>ci-c-spec-134</v>
       </c>
       <c r="P184" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="185" spans="1:16" ht="68" x14ac:dyDescent="0.2">
       <c r="A185" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="B185" s="7" t="s">
         <v>628</v>
       </c>
-      <c r="B185" s="7" t="s">
+      <c r="C185" s="8" t="s">
         <v>629</v>
-      </c>
-      <c r="C185" s="8" t="s">
-        <v>630</v>
       </c>
       <c r="D185" s="7" t="s">
         <v>26</v>
@@ -10262,15 +10263,15 @@
         <v>ci-c-spec-135</v>
       </c>
       <c r="P185" s="10" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="186" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A186" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="B186" s="7" t="s">
         <v>631</v>
-      </c>
-      <c r="B186" s="7" t="s">
-        <v>632</v>
       </c>
       <c r="C186" s="8" t="s">
         <v>39</v>
@@ -10293,18 +10294,18 @@
         <v>ci-c-spec-136</v>
       </c>
       <c r="P186" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="187" spans="1:16" ht="136" x14ac:dyDescent="0.2">
       <c r="A187" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="B187" s="7" t="s">
         <v>633</v>
       </c>
-      <c r="B187" s="7" t="s">
+      <c r="C187" s="8" t="s">
         <v>634</v>
-      </c>
-      <c r="C187" s="8" t="s">
-        <v>635</v>
       </c>
       <c r="D187" s="7" t="s">
         <v>26</v>
@@ -10324,18 +10325,18 @@
         <v>ci-c-spec-137</v>
       </c>
       <c r="P187" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="188" spans="1:16" ht="85" x14ac:dyDescent="0.2">
       <c r="A188" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="B188" s="7" t="s">
         <v>636</v>
       </c>
-      <c r="B188" s="7" t="s">
+      <c r="C188" s="8" t="s">
         <v>637</v>
-      </c>
-      <c r="C188" s="8" t="s">
-        <v>638</v>
       </c>
       <c r="D188" s="7" t="s">
         <v>26</v>
@@ -10355,18 +10356,18 @@
         <v>ci-c-spec-138</v>
       </c>
       <c r="P188" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="189" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="189" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" s="7" t="s">
+        <v>638</v>
+      </c>
+      <c r="B189" s="7" t="s">
         <v>639</v>
       </c>
-      <c r="B189" s="7" t="s">
+      <c r="C189" s="8" t="s">
         <v>640</v>
-      </c>
-      <c r="C189" s="8" t="s">
-        <v>641</v>
       </c>
       <c r="D189" s="7" t="s">
         <v>26</v>
@@ -10386,18 +10387,18 @@
         <v>ci-c-spec-139</v>
       </c>
       <c r="P189" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="190" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="190" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="B190" s="7" t="s">
         <v>642</v>
       </c>
-      <c r="B190" s="7" t="s">
+      <c r="C190" s="8" t="s">
         <v>643</v>
-      </c>
-      <c r="C190" s="8" t="s">
-        <v>644</v>
       </c>
       <c r="D190" s="7" t="s">
         <v>26</v>
@@ -10417,18 +10418,18 @@
         <v>ci-c-spec-140</v>
       </c>
       <c r="P190" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="191" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="191" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A191" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="B191" s="7" t="s">
         <v>645</v>
       </c>
-      <c r="B191" s="7" t="s">
+      <c r="C191" s="8" t="s">
         <v>646</v>
-      </c>
-      <c r="C191" s="8" t="s">
-        <v>647</v>
       </c>
       <c r="D191" s="7" t="s">
         <v>26</v>
@@ -10448,15 +10449,15 @@
         <v>ci-c-spec-141</v>
       </c>
       <c r="P191" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="192" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A192" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="B192" s="7" t="s">
         <v>648</v>
-      </c>
-      <c r="B192" s="7" t="s">
-        <v>649</v>
       </c>
       <c r="C192" s="8" t="s">
         <v>40</v>
@@ -10479,15 +10480,15 @@
         <v>ci-c-spec-142</v>
       </c>
       <c r="P192" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="193" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A193" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="B193" s="7" t="s">
         <v>650</v>
-      </c>
-      <c r="B193" s="7" t="s">
-        <v>651</v>
       </c>
       <c r="C193" s="8" t="s">
         <v>41</v>
@@ -10510,21 +10511,21 @@
         <v>ci-c-spec-143</v>
       </c>
       <c r="P193" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="194" spans="1:16" ht="119" x14ac:dyDescent="0.2">
       <c r="A194" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="B194" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="B194" s="7" t="s">
+      <c r="C194" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="C194" s="8" t="s">
+      <c r="D194" s="7" t="s">
         <v>654</v>
-      </c>
-      <c r="D194" s="7" t="s">
-        <v>655</v>
       </c>
       <c r="E194" s="8" t="s">
         <v>91</v>
@@ -10541,18 +10542,18 @@
         <v>ci-c-spec-144</v>
       </c>
       <c r="P194" s="10" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="195" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A195" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="B195" s="7" t="s">
         <v>656</v>
       </c>
-      <c r="B195" s="7" t="s">
+      <c r="C195" s="8" t="s">
         <v>657</v>
-      </c>
-      <c r="C195" s="8" t="s">
-        <v>658</v>
       </c>
       <c r="D195" s="7" t="s">
         <v>31</v>
@@ -10572,18 +10573,18 @@
         <v>ci-c-spec-145</v>
       </c>
       <c r="P195" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="196" spans="1:16" ht="68" x14ac:dyDescent="0.2">
       <c r="A196" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="B196" s="7" t="s">
         <v>659</v>
       </c>
-      <c r="B196" s="7" t="s">
+      <c r="C196" s="8" t="s">
         <v>660</v>
-      </c>
-      <c r="C196" s="8" t="s">
-        <v>661</v>
       </c>
       <c r="D196" s="7" t="s">
         <v>31</v>
@@ -10603,18 +10604,18 @@
         <v>ci-c-spec-146</v>
       </c>
       <c r="P196" s="10" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="197" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="197" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="B197" s="7" t="s">
         <v>662</v>
       </c>
-      <c r="B197" s="7" t="s">
+      <c r="C197" s="8" t="s">
         <v>663</v>
-      </c>
-      <c r="C197" s="8" t="s">
-        <v>664</v>
       </c>
       <c r="D197" s="7" t="s">
         <v>26</v>
@@ -10634,18 +10635,18 @@
         <v>ci-c-spec-147</v>
       </c>
       <c r="P197" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="198" spans="1:16" ht="136" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="198" spans="1:16" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="B198" s="7" t="s">
         <v>665</v>
       </c>
-      <c r="B198" s="7" t="s">
+      <c r="C198" s="8" t="s">
         <v>666</v>
-      </c>
-      <c r="C198" s="8" t="s">
-        <v>667</v>
       </c>
       <c r="D198" s="7" t="s">
         <v>30</v>
@@ -10665,18 +10666,18 @@
         <v>ci-c-spec-148</v>
       </c>
       <c r="P198" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="199" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="199" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" s="7" t="s">
+        <v>667</v>
+      </c>
+      <c r="B199" s="7" t="s">
         <v>668</v>
       </c>
-      <c r="B199" s="7" t="s">
+      <c r="C199" s="8" t="s">
         <v>669</v>
-      </c>
-      <c r="C199" s="8" t="s">
-        <v>670</v>
       </c>
       <c r="D199" s="7" t="s">
         <v>30</v>
@@ -10696,18 +10697,18 @@
         <v>ci-c-spec-149</v>
       </c>
       <c r="P199" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="200" spans="1:16" ht="85" x14ac:dyDescent="0.2">
       <c r="A200" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="B200" s="7" t="s">
         <v>671</v>
       </c>
-      <c r="B200" s="7" t="s">
+      <c r="C200" s="8" t="s">
         <v>672</v>
-      </c>
-      <c r="C200" s="8" t="s">
-        <v>673</v>
       </c>
       <c r="D200" s="7" t="s">
         <v>26</v>
@@ -10727,18 +10728,18 @@
         <v>ci-c-spec-150</v>
       </c>
       <c r="P200" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="201" spans="1:16" ht="85" x14ac:dyDescent="0.2">
       <c r="A201" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="B201" s="7" t="s">
         <v>674</v>
       </c>
-      <c r="B201" s="7" t="s">
+      <c r="C201" s="8" t="s">
         <v>675</v>
-      </c>
-      <c r="C201" s="8" t="s">
-        <v>676</v>
       </c>
       <c r="D201" s="7" t="s">
         <v>26</v>
@@ -10758,18 +10759,18 @@
         <v>ci-c-spec-151</v>
       </c>
       <c r="P201" s="10" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="202" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A202" s="7" t="s">
+        <v>676</v>
+      </c>
+      <c r="B202" s="7" t="s">
         <v>677</v>
       </c>
-      <c r="B202" s="7" t="s">
+      <c r="C202" s="8" t="s">
         <v>678</v>
-      </c>
-      <c r="C202" s="8" t="s">
-        <v>679</v>
       </c>
       <c r="D202" s="7" t="s">
         <v>26</v>
@@ -10789,18 +10790,18 @@
         <v>ci-c-spec-152</v>
       </c>
       <c r="P202" s="10" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="203" spans="1:16" ht="68" x14ac:dyDescent="0.2">
       <c r="A203" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="B203" s="7" t="s">
         <v>680</v>
       </c>
-      <c r="B203" s="7" t="s">
+      <c r="C203" s="8" t="s">
         <v>681</v>
-      </c>
-      <c r="C203" s="8" t="s">
-        <v>682</v>
       </c>
       <c r="D203" s="7" t="s">
         <v>26</v>
@@ -10820,18 +10821,18 @@
         <v>ci-c-spec-153</v>
       </c>
       <c r="P203" s="10" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="204" spans="1:16" ht="204" x14ac:dyDescent="0.2">
       <c r="A204" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="B204" s="7" t="s">
         <v>683</v>
       </c>
-      <c r="B204" s="7" t="s">
+      <c r="C204" s="8" t="s">
         <v>684</v>
-      </c>
-      <c r="C204" s="8" t="s">
-        <v>685</v>
       </c>
       <c r="D204" s="7" t="s">
         <v>26</v>
@@ -10851,18 +10852,18 @@
         <v>ci-c-spec-154</v>
       </c>
       <c r="P204" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="205" spans="1:16" ht="136" x14ac:dyDescent="0.2">
       <c r="A205" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="B205" s="7" t="s">
         <v>686</v>
       </c>
-      <c r="B205" s="7" t="s">
+      <c r="C205" s="8" t="s">
         <v>687</v>
-      </c>
-      <c r="C205" s="8" t="s">
-        <v>688</v>
       </c>
       <c r="D205" s="7" t="s">
         <v>26</v>
@@ -10882,18 +10883,18 @@
         <v>ci-c-spec-155</v>
       </c>
       <c r="P205" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="206" spans="1:16" ht="119" x14ac:dyDescent="0.2">
       <c r="A206" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="B206" s="7" t="s">
         <v>689</v>
       </c>
-      <c r="B206" s="7" t="s">
+      <c r="C206" s="8" t="s">
         <v>690</v>
-      </c>
-      <c r="C206" s="8" t="s">
-        <v>691</v>
       </c>
       <c r="D206" s="7" t="s">
         <v>26</v>
@@ -10913,18 +10914,18 @@
         <v>ci-c-spec-156</v>
       </c>
       <c r="P206" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="207" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A207" s="7" t="s">
+        <v>691</v>
+      </c>
+      <c r="B207" s="7" t="s">
         <v>692</v>
       </c>
-      <c r="B207" s="7" t="s">
+      <c r="C207" s="8" t="s">
         <v>693</v>
-      </c>
-      <c r="C207" s="8" t="s">
-        <v>694</v>
       </c>
       <c r="D207" s="7" t="s">
         <v>26</v>
@@ -10944,18 +10945,18 @@
         <v>ci-c-spec-157</v>
       </c>
       <c r="P207" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="208" spans="1:16" ht="68" x14ac:dyDescent="0.2">
       <c r="A208" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="B208" s="7" t="s">
         <v>695</v>
       </c>
-      <c r="B208" s="7" t="s">
+      <c r="C208" s="8" t="s">
         <v>696</v>
-      </c>
-      <c r="C208" s="8" t="s">
-        <v>697</v>
       </c>
       <c r="D208" s="7" t="s">
         <v>26</v>
@@ -10975,18 +10976,18 @@
         <v>ci-c-spec-158</v>
       </c>
       <c r="P208" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="209" spans="1:16" ht="221" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="209" spans="1:16" ht="221" hidden="1" x14ac:dyDescent="0.2">
       <c r="A209" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="B209" s="7" t="s">
         <v>698</v>
       </c>
-      <c r="B209" s="7" t="s">
+      <c r="C209" s="8" t="s">
         <v>699</v>
-      </c>
-      <c r="C209" s="8" t="s">
-        <v>700</v>
       </c>
       <c r="D209" s="7" t="s">
         <v>26</v>
@@ -11006,18 +11007,18 @@
         <v>ci-c-spec-159</v>
       </c>
       <c r="P209" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="210" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="210" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="B210" s="7" t="s">
         <v>701</v>
       </c>
-      <c r="B210" s="7" t="s">
+      <c r="C210" s="8" t="s">
         <v>702</v>
-      </c>
-      <c r="C210" s="8" t="s">
-        <v>703</v>
       </c>
       <c r="D210" s="7" t="s">
         <v>26</v>
@@ -11037,18 +11038,18 @@
         <v>ci-c-spec-160</v>
       </c>
       <c r="P210" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="211" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="211" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="B211" s="7" t="s">
         <v>704</v>
       </c>
-      <c r="B211" s="7" t="s">
+      <c r="C211" s="8" t="s">
         <v>705</v>
-      </c>
-      <c r="C211" s="8" t="s">
-        <v>706</v>
       </c>
       <c r="D211" s="7" t="s">
         <v>30</v>
@@ -11068,18 +11069,18 @@
         <v>ci-c-spec-161</v>
       </c>
       <c r="P211" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="212" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="212" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="B212" s="7" t="s">
         <v>707</v>
       </c>
-      <c r="B212" s="7" t="s">
+      <c r="C212" s="8" t="s">
         <v>708</v>
-      </c>
-      <c r="C212" s="8" t="s">
-        <v>709</v>
       </c>
       <c r="D212" s="7" t="s">
         <v>29</v>
@@ -11099,21 +11100,21 @@
         <v>ci-c-spec-162</v>
       </c>
       <c r="P212" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="213" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="213" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="B213" s="7" t="s">
         <v>710</v>
       </c>
-      <c r="B213" s="7" t="s">
+      <c r="C213" s="8" t="s">
         <v>711</v>
       </c>
-      <c r="C213" s="8" t="s">
+      <c r="D213" s="7" t="s">
         <v>712</v>
-      </c>
-      <c r="D213" s="7" t="s">
-        <v>713</v>
       </c>
       <c r="E213" s="8" t="s">
         <v>91</v>
@@ -11130,18 +11131,18 @@
         <v>ci-c-spec-163</v>
       </c>
       <c r="P213" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="214" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="214" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" s="7" t="s">
+        <v>713</v>
+      </c>
+      <c r="B214" s="7" t="s">
         <v>714</v>
       </c>
-      <c r="B214" s="7" t="s">
+      <c r="C214" s="8" t="s">
         <v>715</v>
-      </c>
-      <c r="C214" s="8" t="s">
-        <v>716</v>
       </c>
       <c r="D214" s="7" t="s">
         <v>29</v>
@@ -11161,18 +11162,18 @@
         <v>ci-c-spec-164</v>
       </c>
       <c r="P214" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="215" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="215" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="B215" s="7" t="s">
         <v>717</v>
       </c>
-      <c r="B215" s="7" t="s">
+      <c r="C215" s="8" t="s">
         <v>718</v>
-      </c>
-      <c r="C215" s="8" t="s">
-        <v>719</v>
       </c>
       <c r="D215" s="7" t="s">
         <v>31</v>
@@ -11192,18 +11193,18 @@
         <v>ci-c-spec-165</v>
       </c>
       <c r="P215" s="10" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="216" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="216" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="B216" s="7" t="s">
         <v>720</v>
       </c>
-      <c r="B216" s="7" t="s">
+      <c r="C216" s="8" t="s">
         <v>721</v>
-      </c>
-      <c r="C216" s="8" t="s">
-        <v>722</v>
       </c>
       <c r="D216" s="7" t="s">
         <v>30</v>
@@ -11223,15 +11224,32 @@
         <v>ci-c-spec-166</v>
       </c>
       <c r="P216" s="10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE216" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}"/>
+  <autoFilter ref="A1:AE216" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="SHALL"/>
+        <filter val="SHALL / MAY"/>
+        <filter val="SHALL / SHOULD"/>
+        <filter val="SHALL NOT"/>
+        <filter val="SHALL NOT / MAY"/>
+        <filter val="SHALL NOT / SHALL"/>
+        <filter val="SHALL NOT / SHOULD"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="DTR Client"/>
+        <filter val="DTR Client, DTR Server"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" location="ci-c-conf-5" xr:uid="{54FDFC2F-0C71-9847-9311-57A99C2A2FC8}"/>
-    <hyperlink ref="B40" r:id="rId2" location="ci-c-prof-2" xr:uid="{7290C952-57E1-8842-B595-0231F7C148ED}"/>
-    <hyperlink ref="B64" r:id="rId3" location="ci-c-spec-14" xr:uid="{00DAE728-E8A3-4041-ABBD-1CA449CC91CF}"/>
+    <hyperlink ref="B25" r:id="rId1" location="ci-c-oper-7" xr:uid="{4023679D-7765-2B42-A707-2B63CD4C2439}"/>
+    <hyperlink ref="B75" r:id="rId2" location="ci-c-spec-25" xr:uid="{C6E51CB5-4ECD-3246-931F-4ABAFB05C0AF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>